<commit_message>
feat: add global announcement ribbon powered by Google Sheet
</commit_message>
<xml_diff>
--- a/Arena_2026_Data.xlsx
+++ b/Arena_2026_Data.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="106">
   <si>
     <t>key</t>
   </si>
@@ -94,6 +94,9 @@
   </si>
   <si>
     <t>Delhi Technological University</t>
+  </si>
+  <si>
+    <t>announcement_ribbon_text</t>
   </si>
   <si>
     <t>dept_id</t>
@@ -726,10 +729,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="23" customWidth="1"/>
+    <col min="1" max="1" width="27" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
   </cols>
   <sheetData>
@@ -835,6 +838,14 @@
       </c>
       <c r="B13" t="s">
         <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -853,13 +864,13 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -879,27 +890,27 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C2" t="s">
         <v>21</v>
@@ -908,15 +919,15 @@
         <v>21</v>
       </c>
       <c r="E2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
         <v>21</v>
@@ -925,15 +936,15 @@
         <v>21</v>
       </c>
       <c r="E3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C4" t="s">
         <v>21</v>
@@ -942,15 +953,15 @@
         <v>21</v>
       </c>
       <c r="E4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C5" t="s">
         <v>21</v>
@@ -959,15 +970,15 @@
         <v>21</v>
       </c>
       <c r="E5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C6" t="s">
         <v>21</v>
@@ -976,15 +987,15 @@
         <v>21</v>
       </c>
       <c r="E6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C7" t="s">
         <v>21</v>
@@ -993,15 +1004,15 @@
         <v>21</v>
       </c>
       <c r="E7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C8" t="s">
         <v>21</v>
@@ -1010,15 +1021,15 @@
         <v>21</v>
       </c>
       <c r="E8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C9" t="s">
         <v>21</v>
@@ -1027,15 +1038,15 @@
         <v>21</v>
       </c>
       <c r="E9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C10" t="s">
         <v>21</v>
@@ -1044,7 +1055,7 @@
         <v>21</v>
       </c>
       <c r="E10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1064,19 +1075,19 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -1095,43 +1106,43 @@
   <sheetData>
     <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1152,19 +1163,19 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1183,13 +1194,13 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1208,10 +1219,10 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -1232,86 +1243,86 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update official tournament games list and required player quotas
</commit_message>
<xml_diff>
--- a/Arena_2026_Data.xlsx
+++ b/Arena_2026_Data.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="118">
   <si>
     <t>key</t>
   </si>
@@ -117,16 +117,106 @@
     <t>has_girls</t>
   </si>
   <si>
+    <t>nos_of_players</t>
+  </si>
+  <si>
     <t>display_order</t>
   </si>
   <si>
+    <t>cricket</t>
+  </si>
+  <si>
+    <t>Cricket</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>Man-15, Women-8</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>football</t>
+  </si>
+  <si>
+    <t>Football</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
     <t>basketball</t>
   </si>
   <si>
     <t>Basketball</t>
   </si>
   <si>
-    <t>1</t>
+    <t>Man-8, Women-6</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>volleyball</t>
+  </si>
+  <si>
+    <t>Volleyball</t>
+  </si>
+  <si>
+    <t>Man-10, Women-(6-8)</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>kabaddi</t>
+  </si>
+  <si>
+    <t>Kabaddi</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>lawn-tennis</t>
+  </si>
+  <si>
+    <t>Lawn Tennis</t>
+  </si>
+  <si>
+    <t>Open to all</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>athletics</t>
+  </si>
+  <si>
+    <t>Athletics</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>badminton</t>
+  </si>
+  <si>
+    <t>Badminton</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>chess</t>
+  </si>
+  <si>
+    <t>Chess</t>
+  </si>
+  <si>
+    <t>9</t>
   </si>
   <si>
     <t>table-tennis</t>
@@ -135,70 +225,16 @@
     <t>Table Tennis</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>kabaddi</t>
-  </si>
-  <si>
-    <t>Kabaddi</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>football</t>
-  </si>
-  <si>
-    <t>Football</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>volleyball</t>
-  </si>
-  <si>
-    <t>Volleyball</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>cricket</t>
-  </si>
-  <si>
-    <t>Cricket</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>badminton</t>
-  </si>
-  <si>
-    <t>Badminton</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>chess</t>
-  </si>
-  <si>
-    <t>Chess</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>hockey</t>
-  </si>
-  <si>
-    <t>Hockey</t>
-  </si>
-  <si>
-    <t>9</t>
+    <t>10</t>
+  </si>
+  <si>
+    <t>carom</t>
+  </si>
+  <si>
+    <t>Carom (Mixed)</t>
+  </si>
+  <si>
+    <t>11</t>
   </si>
   <si>
     <t>category</t>
@@ -881,14 +917,17 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -904,158 +943,228 @@
       <c r="E1" s="1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="E2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+      <c r="F2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" t="s">
         <v>37</v>
       </c>
-      <c r="C3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="E4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+      <c r="F4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B5" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="E5" t="s">
+        <v>48</v>
+      </c>
+      <c r="F5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B7" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="E7" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+      <c r="F7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="B8" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="E8" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+      <c r="F8" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9" t="s">
         <v>55</v>
       </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="D10" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="E10" t="s">
-        <v>59</v>
+        <v>55</v>
+      </c>
+      <c r="F10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" t="s">
+        <v>36</v>
+      </c>
+      <c r="E11" t="s">
+        <v>55</v>
+      </c>
+      <c r="F11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>69</v>
+      </c>
+      <c r="B12" t="s">
+        <v>70</v>
+      </c>
+      <c r="C12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" t="s">
+        <v>36</v>
+      </c>
+      <c r="E12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F12" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1081,13 +1190,13 @@
         <v>29</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1106,43 +1215,43 @@
   <sheetData>
     <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -1166,16 +1275,16 @@
         <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -1194,13 +1303,13 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1219,10 +1328,10 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1243,86 +1352,86 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="B2" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="C2" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="D2" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="B3" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="C3" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="D3" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="B4" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="C4" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="D4" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="B5" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="C5" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="D5" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="B6" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="C6" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="D6" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>